<commit_message>
Replace questions 20, 23 and 24 and extend Q1's explanation
The owner revised the bank: new Q20 (petroleum operations), Q23
(royalty exemption) and Q24 (statutes preserving the concession); the
former Q24 moves to Q22 unchanged; the former Q20, Q22 and Q23 are
removed; Q1's explanation gains a closing sentence. Levels are now
4 foundational, 9 intermediate and 12 advanced.

- data/questions.xlsx follows the owner's new 8-column layout (السؤال,
  السند النظامي, options separated by ؛), plus the guide sheet.
- build_questions.py accepts the السؤال header and ؛-separated options
  as well as the previous layout.
- Storage key v4 so progress saved against the previous numbering is
  ignored; asset version tags bumped; README updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdJRTf8G26dx7ZenTkKWdk
</commit_message>
<xml_diff>
--- a/data/questions.xlsx
+++ b/data/questions.xlsx
@@ -11,7 +11,7 @@
     <sheet name="طريقة التعبئة" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بنك الأسئلة'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بنك الأسئلة'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,11 +41,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001F5C99"/>
       <sz val="10"/>
     </font>
     <font>
@@ -115,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -132,9 +127,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
@@ -145,9 +137,6 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,10 +151,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
@@ -537,18 +523,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="62" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -569,30 +554,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>محور القياس</t>
+          <t>السؤال</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>نص السؤال</t>
+          <t>الخيارات</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>الخيارات</t>
+          <t>الإجابة الصحيحة</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>الإجابة الصحيحة</t>
+          <t>السند النظامي</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>السند النظامي ذو الارتباط</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>شرح مبسط</t>
         </is>
@@ -612,36 +592,29 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>اختصاص</t>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>لا يُعد من مهام الهيئة السعودية لتنظيم الكهرباء:</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>لا يُعد من مهام الهيئة السعودية لتنظيم الكهرباء:</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>إصدار اللوائح التنفيذية
-البت في الشكاوى المتعلقة بنشاط الكهرباء
-إعداد السياسات والاستراتيجيات الوطنية لقطاع الكهرباء</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
+          <t>إصدار اللوائح التنفيذية ؛ البت في الشكاوى المتعلقة بنشاط الكهرباء ؛ إعداد السياسات والاستراتيجيات الوطنية لقطاع الكهرباء</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>إعداد السياسات والاستراتيجيات الوطنية لقطاع الكهرباء</t>
         </is>
       </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>الفقرة (1) من المادة (3) في اختصاص الوزارة، مقابل المادة (4) في اختصاص الهيئة</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>الفقرة (1) من المادة (3) في اختصاص الوزارة، مقابل المادة (4) في اختصاص الهيئة</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>إعداد السياسات والاستراتيجيات والرفع بها لاعتمادها اختصاص أصيل للوزارة، بينما تعمل الهيئة في ضوء تلك السياسات المعتمدة.</t>
+          <t>إعداد السياسات والاستراتيجيات والرفع بها لاعتمادها اختصاص أصيل للوزارة، بينما تعمل الهيئة في ضوء تلك السياسات المعتمدة. وهذا السؤال يقيس التفريق بين دور صانع السياسة ودور المنظم.</t>
         </is>
       </c>
     </row>
@@ -659,369 +632,307 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>مفهوم</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>الفرق بين "التعريفة" و"السعر" في نظام الكهرباء أن:</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>الفرق بين "التعريفة" و"السعر" في نظام الكهرباء أن:</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>التعريفة مقابل مالي معتمد، والسعر مقابل يُتفق عليه بين مرخص لهما أو بين مرخص له ومستهلك كبير
-التعريفة تشمل الضريبة والسعر لا يشملها
-التعريفة سنوية والسعر يراجع شهرياً
-التعريفة للمستهلك المنزلي والسعر للمستهلك التجاري</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
+          <t>التعريفة مقابل مالي معتمد، والسعر مقابل يُتفق عليه بين مرخص لهما أو بين مرخص له ومستهلك كبير ؛ التعريفة تشمل الضريبة والسعر لا يشملها ؛ التعريفة سنوية والسعر يراجع شهرياً ؛ التعريفة للمستهلك المنزلي والسعر للمستهلك التجاري</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>التعريفة مقابل مالي معتمد، والسعر مقابل يُتفق عليه بين مرخص لهما أو بين مرخص له ومستهلك كبير</t>
         </is>
       </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>المادة (1) - تعريفا التعريفة والسعر، مع الفقرة (3) من المادة (12)</t>
+        </is>
+      </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>المادة (1) - تعريفا التعريفة والسعر، مع الفقرة (3) من المادة (12)</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
           <t>التعريفة معتمدة وتسري على فئات المستهلكين، والسعر ثمرة تفاوض تجاري مباشر يجوز أن يختلف عن التعريفة المعتمدة وفق ما تحدده اللوائح. ولهذا ارتبط وصف المستهلك الكبير بأثر عملي، وهو إمكان التعاقد بسعر خارج التعريفة.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>إجراء ومدة</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>تتخذ الهيئة السعودية لتنظيم الكهرباء إجراءات عاجلة بحق المخالف مثل:</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>إيقاف مزاولة نشاط الكهرباء جزئياً أو كلياً لمدة لا تتجاوز سنة
-إلغاء الرخصة
-إيقاف مزاولته للنشاط جزئياً أو كلياً بما لا يتجاوز (6) أشهر</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>إيقاف مزاولة نشاط الكهرباء جزئياً أو كلياً لمدة لا تتجاوز سنة ؛ إلغاء الرخصة ؛ إيقاف مزاولته للنشاط جزئياً أو كلياً بما لا يتجاوز (6) أشهر</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>إيقاف مزاولته للنشاط جزئياً أو كلياً بما لا يتجاوز (6) أشهر</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (ج) من الفقرة (1) من المادة (20)، مقابل الفقرة (1) من المادة (18)</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>يفرق النظام بين إجراء عاجل تتخذه الهيئة بقرار من المحافظ أو من ينيبه ومدته لا تتجاوز ستة أشهر، وبين عقوبة توقعها اللجنة بعد النظر في المخالفة وتصل إلى إيقاف سنة أو إلغاء الرخصة أو غرامة. والخياران الآخران عقوبات لا إجراءات عاجلة.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>حد ونسبة</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>يجب على المرخص له الحصول على موافقة الهيئة قبل شراء أسهم مرخص له آخر إذا بلغت النسبة:</t>
         </is>
       </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>(10%) عشرة في المائة أو أكثر ؛ (20%) عشرين في المائة أو أكثر ؛ أي نسبة مهما قلّت ؛ (5%) خمسة في المائة أو أكثر، أو نسبة أقل إذا أدت إلى إنشاء وضع مهيمن</t>
+        </is>
+      </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>(10%) عشرة في المائة أو أكثر
-(20%) عشرين في المائة أو أكثر
-أي نسبة مهما قلّت
-(5%) خمسة في المائة أو أكثر، أو نسبة أقل إذا أدت إلى إنشاء وضع مهيمن</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr">
-        <is>
           <t>(5%) خمسة في المائة أو أكثر، أو نسبة أقل إذا أدت إلى إنشاء وضع مهيمن</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>الفقرة (5) من المادة (13)، مع تعريف الوضع المهيمن في المادة (1)</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>العتبة الرقمية خمسة في المائة، ومعها عتبة وصفية مؤداها أن النسبة الأقل تحتاج موافقة كذلك متى أدت إلى إنشاء وضع مهيمن في أي جزء من الأنشطة الكهربائية. والوضع المهيمن معرّف بأنه امتلاك القدرة على التأثير في عدالة اتخاذ القرارات أو التنافس المشروع.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>مهلة ووسيلة تظلم</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>إذا رفضت الهيئة إصدار رخصة لشخص استوفى جميع الشروط، أو مضى (30) يوم عمل من تاريخ اكتمال طلبه دون البت فيه، فله الحق النظامي في:</t>
         </is>
       </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>التظلم أمام المحكمة التجارية ؛ التظلم أمام المحكمة الإدارية ؛ الاعتراض أمام الهيئة السعودية لتنظيم الكهرباء</t>
+        </is>
+      </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>التظلم أمام المحكمة التجارية
-التظلم أمام المحكمة الإدارية
-الاعتراض أمام الهيئة السعودية لتنظيم الكهرباء</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
           <t>التظلم أمام المحكمة الإدارية</t>
         </is>
       </c>
-      <c r="H6" s="13" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>الفقرة (4) من المادة (5)</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>أوجب النظام إصدار الرخصة خلال ثلاثين يوم عمل من اكتمال الطلب متى توافرت الشروط، واشترط تسبيب قرار الرفض، وأتاح لمن رفض طلبه أو مضت المدة دون بت التظلم أمام المحكمة الإدارية. والسبب أن القرار قرار إداري لا نزاع تجاري.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>اختصاص</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>الجهة المختصة بإصدار رخص مزاولة أوجه النشاط بعد تعديل النظام هي:</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>هيئة تنظيم المياه والكهرباء
-وزارة الطاقة
-وزارة الصناعة والثروة المعدنية
-الهيئة العامة للنقل</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>هيئة تنظيم المياه والكهرباء ؛ وزارة الطاقة ؛ وزارة الصناعة والثروة المعدنية ؛ الهيئة العامة للنقل</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>وزارة الطاقة</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>المادة (3) بعد تعديلها بالمرسوم الملكي رقم (م/112) وتاريخ 1443/11/9هـ</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>صدر النظام سنة 1438 وأسند الاختصاص إلى الهيئة، ثم نقله التعديل إلى الوزارة بإحلال كلمة الوزارة محل الهيئة. ولهذا يجب الرجوع إلى النص المعدل لا الأصلي عند تحديد الجهة المختصة.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>حد ورقم</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>تُعد في حكم المستهلك التجاري المنشآت الصناعية الصغيرة التي لا يتجاوز استهلاكها للغاز الجاف:</t>
         </is>
       </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>(176.500) قدم مكعب يومياً ؛ (100.000) قدم مكعب يومياً ؛ (500.000) قدم مكعب يومياً ؛ (250.000) قدم مكعب يومياً</t>
+        </is>
+      </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>(176.500) قدم مكعب يومياً
-(100.000) قدم مكعب يومياً
-(500.000) قدم مكعب يومياً
-(250.000) قدم مكعب يومياً</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
           <t>(176.500) قدم مكعب يومياً</t>
         </is>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>المادة (1) - تعريف المستهلك التجاري</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>الحد رقم منصوص عليه في التعريف نفسه لا تحدده اللوائح، وأثره أن المنشأة الصناعية الصغيرة دون هذا الحد تعامل معاملة المستهلك التجاري وتخضع لهذا النظام، وما تجاوزه يخرج إلى منظومة تخصيص الطاقة.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>مهلة وأثرها</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>تقدم مرخص له بطلب موافقة على نقل ملكية أصول أساسية، ومضت تسعون يوماً من تاريخ اكتمال الطلب دون بت. الأثر النظامي:</t>
         </is>
       </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>يُعد مضي المدة إذناً له بالتصرف ؛ يُعد الطلب مرفوضاً ضمناً ؛ يجب عليه التقدم بطلب جديد ؛ يُحال الطلب إلى اللجنة للنظر فيه</t>
+        </is>
+      </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>يُعد مضي المدة إذناً له بالتصرف
-يُعد الطلب مرفوضاً ضمناً
-يجب عليه التقدم بطلب جديد
-يُحال الطلب إلى اللجنة للنظر فيه</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
           <t>يُعد مضي المدة إذناً له بالتصرف</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>المادة (13) بعد تعديلها بالمرسوم الملكي رقم (م/112)</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>المدة تسعون يوماً من اكتمال الطلب، ورتب النظام على مضيها دون بت أثراً إيجابياً هو الإذن بالتصرف لا الرفض الضمني. ويجب أن يكون قرار الرفض مسبباً. والأصول الأساسية هي ما يترتب على نقل ملكيتها إخلال بأداء النشاط المرخص به، ومنها شبكة توزيع الغاز الجاف ومرافق غاز البترول السائل.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>حد الغرامة</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>الحد الأعلى للغرامة على مخالفة أحكام نظام توزيع الغاز الجاف وغاز البترول السائل هو:</t>
         </is>
       </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>عشرة ملايين ريال ؛ خمسة ملايين ريال ؛ ثلاثون مليون ريال ؛ عشرون مليون ريال</t>
+        </is>
+      </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>عشرة ملايين ريال
-خمسة ملايين ريال
-ثلاثون مليون ريال
-عشرون مليون ريال</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
           <t>خمسة ملايين ريال</t>
         </is>
       </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (أ) من الفقرة (1) من المادة (16)</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>سقف الغرامة هنا خمسة ملايين، ويجوز أن يقترن بإيقاف النشاط جزئياً أو كلياً لمدة لا تتجاوز سنة أو بإلغاء الرخصة. ويفيد استحضار الأسقف في أنظمة القطاع معاً: نظام الكهرباء عشرة ملايين، وإمدادات الطاقة عشرون مليوناً، وجريمة تصدير المادة البترولية المسعرة ثلاثون مليوناً أو ضعفا قيمتها أيهما أعلى.</t>
         </is>
@@ -1041,762 +952,634 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>وصف نظامي</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>أي وصف نظامي يلحق ملكية الدولة للموارد الهيدروكربونية؟</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>أي وصف نظامي يلحق ملكية الدولة للموارد الهيدروكربونية؟</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>غير قابلة للتصرف ولا تسقط بالتقادم
-تنتقل إلى المرخص له بانتهاء مدة الرخصة
-تسقط بالتقادم الطويل إذا لم تستغل
-قابلة للتصرف بموافقة مجلس الوزراء</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+          <t>غير قابلة للتصرف ولا تسقط بالتقادم ؛ تنتقل إلى المرخص له بانتهاء مدة الرخصة ؛ تسقط بالتقادم الطويل إذا لم تستغل ؛ قابلة للتصرف بموافقة مجلس الوزراء</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>غير قابلة للتصرف ولا تسقط بالتقادم</t>
         </is>
       </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>المادة (5) مع المادة (4)</t>
+        </is>
+      </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>المادة (5) مع المادة (4)</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
           <t>حصّن النظام ملكية الدولة بوصفين معاً: عدم قابليتها للتصرف، وعدم سقوطها بالتقادم، فلا يكسب أحد حقاً عليها بطول وضع اليد ولا بتصرف يقع من أي جهة. ويسند ذلك أن للدولة سيادة دائمة على هذه الموارد تمارسها بما يحقق مصلحتها وأمنها وتنميتها الاقتصادية.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>لحظة انتقال الملكية</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>تنتقل ملكية المواد الهيدروكربونية من الدولة إلى المرخص له عند:</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>توقيع الرخصة
-سداد الريع المستحق عن الكمية المنتجة
-تصدير المنتج خارج الإقليم
-رأس البئر، أو عند استخلاصها في منشأة معالجة لتحصيل منتجات القطران الطبيعي ورمال القار وما في حكمها</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>توقيع الرخصة ؛ سداد الريع المستحق عن الكمية المنتجة ؛ تصدير المنتج خارج الإقليم ؛ رأس البئر، أو عند استخلاصها في منشأة معالجة لتحصيل منتجات القطران الطبيعي ورمال القار وما في حكمها</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>رأس البئر، أو عند استخلاصها في منشأة معالجة لتحصيل منتجات القطران الطبيعي ورمال القار وما في حكمها</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>المادة (3)</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>النظام حدد نقطة زمنية ومكانية لانتقال الملكية، وهي رأس البئر في الحالة المعتادة، أو لحظة الاستخلاص في منشأة المعالجة في حالات القطران الطبيعي وأحجار أو رمال القار وغيرها من مواد الصخور. وقبل هذه النقطة المادة ملك للدولة، فالرخصة تمنح حق ممارسة العمليات لا ملكية الثروة في باطن الأرض.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>مفهوم</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>المقصود بـ "قرار الإنتاج" في النظام هو:</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>قرار يصدر عن منظمة أوبك وتلتزم به المملكة
-خطة تشغيلية سنوية يعدها المرخص له
-قرار تجاري تتخذه الشركة المنتجة بحسب أسعار السوق
-أمر أو توجيه مكتوب من الدولة يضع الحد الأقصى للإنتاج أو يحدد مستوى الطاقة الإنتاجية القصوى المستدامة</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>قرار يصدر عن منظمة أوبك وتلتزم به المملكة ؛ خطة تشغيلية سنوية يعدها المرخص له ؛ قرار تجاري تتخذه الشركة المنتجة بحسب أسعار السوق ؛ أمر أو توجيه مكتوب من الدولة يضع الحد الأقصى للإنتاج أو يحدد مستوى الطاقة الإنتاجية القصوى المستدامة</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>أمر أو توجيه مكتوب من الدولة يضع الحد الأقصى للإنتاج أو يحدد مستوى الطاقة الإنتاجية القصوى المستدامة</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>المادة (1) - التعريفات، والمادة (7)</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>قرار الإنتاج أداة سيادية لا تجارية، وتراعي الدولة عند اتخاذه اعتبارات التنمية الاقتصادية والبيئة والأمن الوطني والسياسة الخارجية والاحتياجات المحلية للطاقة والمصلحة العامة.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>قيد واستثناء</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>متى يُمنع المرخص له من بيع مادة هيدروكربونية أو مشتق منها حصل عليه بموجب الرخصة؟</t>
         </is>
       </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>إذا كان المشتري شخصاً أجنبياً ؛ إذا خالف البيع ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا للدولة في وقت الحرب أو في الحالات الطارئة في العلاقات الدولية ؛ إذا لم تصادق الوزارة على عقد البيع مسبقاً ؛ إذا قل سعر البيع عن السعر العالمي وقت التعاقد</t>
+        </is>
+      </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>إذا كان المشتري شخصاً أجنبياً
-إذا خالف البيع ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا للدولة في وقت الحرب أو في الحالات الطارئة في العلاقات الدولية
-إذا لم تصادق الوزارة على عقد البيع مسبقاً
-إذا قل سعر البيع عن السعر العالمي وقت التعاقد</t>
-        </is>
-      </c>
-      <c r="G14" s="16" t="inlineStr">
-        <is>
           <t>إذا خالف البيع ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا للدولة في وقت الحرب أو في الحالات الطارئة في العلاقات الدولية</t>
         </is>
       </c>
-      <c r="H14" s="13" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>نص النظام في شأن قيد البيع لحماية مصالح الأمن العليا للدولة</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>القيد استثنائي ومربوط بحالتين: وقت الحرب، والحالات الطارئة في العلاقات الدولية، ومناطه ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا. فهو ليس قيداً على هوية المشتري ولا على السعر ولا رقابة مسبقة على العقود.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>اختصاص</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>أي مما يلي لا يُعد من مهام لجنة تخصيص الطاقة؟</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>اعتماد معايير تخصيص الطاقة التي تقترحها الوزارة
-إعداد لائحة التخصيص واقتراح تعديلها
-مراجعة معايير التخصيص كل ثلاث سنوات أو حسب الحاجة
-إصدار وثيقة تخصيص الطاقة للمستهلك</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>اعتماد معايير تخصيص الطاقة التي تقترحها الوزارة ؛ إعداد لائحة التخصيص واقتراح تعديلها ؛ مراجعة معايير التخصيص كل ثلاث سنوات أو حسب الحاجة ؛ إصدار وثيقة تخصيص الطاقة للمستهلك</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>إصدار وثيقة تخصيص الطاقة للمستهلك</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>الفقرة (3) من المادة (3)، مقابل المادة (4)</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>اللجنة جهة معايير وسياسات، أما الإصدار الفعلي لوثيقة التخصيص فتقوم به الوزارة بناءً على الطاقة المتاحة والمعايير المعتمدة من اللجنة. والتفريق بين من يضع المعيار ومن يطبقه هو مربط السؤال.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>نطاق الترخيص</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>أي مما يلي لا يدخل ضمن الأنشطة التي يشترط لها ترخيص من الوزارة بموجب نظام إمدادات الطاقة؟</t>
         </is>
       </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>تنقية الغاز ؛ تكرير الزيت الخام ؛ تجميع الغاز الطبيعي وسوائله ؛ التوزيع المحلي للغاز الطبيعي وسوائله</t>
+        </is>
+      </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>تنقية الغاز
-تكرير الزيت الخام
-تجميع الغاز الطبيعي وسوائله
-التوزيع المحلي للغاز الطبيعي وسوائله</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
           <t>تكرير الزيت الخام</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>الفقرة (1) من المادة (5)، مقابل الفقرة (1) من المادة (2)</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>الترخيص في هذا النظام مقصور على أنشطة الغاز الطبيعي وسوائله والأنشطة المتعلقة بالهيدروجين، وتشمل النقل والمعالجة والتجزئة وتنقية الغاز والتجميع والتخزين والتوزيع المحلي والاستيراد والتصدير والبيع وإنشاء وتملك وتشغيل الشبكات والمرافق. أما تكرير الزيت الخام فهو مجال من مجالات تخصيص الطاقة لا نشاط مرخص بهذا النظام، وتحكمه منظومة المواد البترولية والبتروكيماوية.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>توقيت إجرائي</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>يشترط الحصول على وثيقة تخصيص الطاقة من الوزارة:</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>قبل صدور موافقة الجهة المشرفة بممارسة النشاط الذي يتطلب تخصيصاً للطاقة
-بعد بدء التشغيل الفعلي
-عند تجديد السجل التجاري
-عند تصدير المنتج إلى خارج المملكة</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>قبل صدور موافقة الجهة المشرفة بممارسة النشاط الذي يتطلب تخصيصاً للطاقة ؛ بعد بدء التشغيل الفعلي ؛ عند تجديد السجل التجاري ؛ عند تصدير المنتج إلى خارج المملكة</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>قبل صدور موافقة الجهة المشرفة بممارسة النشاط الذي يتطلب تخصيصاً للطاقة</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>المادة (6)</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>جعل النظام وثيقة التخصيص شرطاً سابقاً على موافقة الجهة المشرفة، حتى لا تُمنح تراخيص لمشاريع لا تتوافر لها طاقة مخصصة. وهذا من أهم الآثار العملية للنظام على المستثمرين.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>حد الغرامة</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>الحد الأعلى للغرامة على مخالفة أحكام النظام أو اللوائح أو لائحة التخصيص أو التراخيص هو:</t>
         </is>
       </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>عشرة ملايين ريال ؛ عشرون مليون ريال ؛ ثلاثون مليون ريال ؛ خمسة ملايين ريال</t>
+        </is>
+      </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>عشرة ملايين ريال
-عشرون مليون ريال
-ثلاثون مليون ريال
-خمسة ملايين ريال</t>
-        </is>
-      </c>
-      <c r="G18" s="16" t="inlineStr">
-        <is>
           <t>عشرون مليون ريال</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (أ) من الفقرة (1) من المادة (8)</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>تصل الغرامة إلى عشرين مليون ريال، ويجوز معها إيقاف الترخيص جزئياً أو كلياً لمدة لا تتجاوز سنة، أو إلغاؤه. ويقابل ذلك سقف مماثل لمخالفة وثيقة التخصيص.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>تنازع نطاق</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>أي نظام يحكم نقل المواد البترولية وتخزينها واستيرادها وتصديرها؟</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>نظام إمدادات الطاقة
-نظام المواد البترولية والبتروكيماوية
-نظام المواد الهيدروكربونية
-نظام توزيع الغاز الجاف وغاز البترول السائل</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>نظام إمدادات الطاقة ؛ نظام المواد البترولية والبتروكيماوية ؛ نظام المواد الهيدروكربونية ؛ نظام توزيع الغاز الجاف وغاز البترول السائل</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>المادة (1) - تعريف العمليات البترولية، مقابل المادة (1) من نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>النظامان يقتسمان سلسلة القيمة: المواد الهيدروكربونية يحكم المنبع من مسح وكشف وتنقيب وحفر وتقييم وتطوير واستخراج وإنتاج ومعالجة، والمواد البترولية والبتروكيماوية يحكم المصب من استخدام وبيع وشراء ونقل وتخزين واستيراد وتصدير وتعبئة، ويدخل فيه إنشاء أو تشغيل مصفاة تكرير أو فرضة أو محطة توزيع. وتحديد النظام الحاكم هو أول ما يُسأل عنه المستشار في أي معاملة.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>إلغاء وإحلال</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>النظام الذي حل محله نظام المواد البترولية والبتروكيماوية هو:</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>نظام المواد الهيدروكربونية
-نظام التجارة بالمنتجات البترولية
-نظام إمدادات الغاز وتسعيره
-نظام الكهرباء</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>نظام المواد الهيدروكربونية ؛ نظام التجارة بالمنتجات البترولية ؛ نظام إمدادات الغاز وتسعيره ؛ نظام الكهرباء</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>نظام التجارة بالمنتجات البترولية</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>المادة (21)</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>حل النظام محل نظام التجارة بالمنتجات البترولية الصادر في 28 محرم 1439هـ، وألغى ما يتعارض معه من أحكام. أما نظام المواد الهيدروكربونية فباق ويغطي مرحلة المنبع.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>الأول (تأسيسي)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>أي مما يلي لا يدخل ضمن العمليات البترولية كما عرفها النظام؟</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>تخزين المواد البترولية أو استيرادها أو تصديرها ؛ بيع المواد البترولية أو شراؤها أو نقلها ؛ التنقيب عن الزيت الخام واستخراجه ؛ إنشاء أو تشغيل مصفاة تكرير أو محطة توزيع</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>التنقيب عن الزيت الخام واستخراجه</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>المادة (1) - تعريف العمليات البترولية</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>العمليات البترولية في هذا النظام تقع في المصب: الاستخدام والبيع والشراء والنقل والتخزين والاستيراد والتصدير والتعبئة والمعالجة وإنشاء المصافي والفرض ومحطات التوزيع. أما التنقيب والاستخراج فمحلهما نظام المواد الهيدروكربونية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>نظام المواد البترولية والبتروكيماوية</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>المتقدم</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>عقوبة من صدّر إلى خارج المملكة مادة بترولية مسعرة دون ترخيص أو شرع في ذلك تشمل:</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>الإنذار ثم الغرامة ؛ الغرامة فقط ؛ إلغاء الترخيص فقط ؛ السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>المادة (15)</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>هذه من أشد العقوبات في أنظمة قطاع الطاقة لأنها تمس الدعم الحكومي للمواد المسعرة، ولذلك جمعت بين السجن والغرامة والمصادرة، وجعلت الغرامة مرتبطة بقيمة المادة بالسعر العالمي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>اتفاقية الامتياز</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>المتقدم</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>أي مما يلي لا يُستحق عليه ريع بموجب اتفاقية الامتياز؟</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها ؛ سوائل الغاز المباعة للغير ؛ الزيت الخام الذي تستخدمه الشركة في عملياتها ؛ المكثفات المنتجة</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>الفقرتان (أ) و(ب) من المادة (7-1) من الاتفاقية</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>الاتفاقية فرّقت بين الزيت والغاز في معاملة الاستخدام الذاتي: ريع الزيت الخام والمكثفات يشمل ما تستخدمه الشركة في عملياتها، أما الغاز وسوائله فلا ريع على ما يُستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها من معامل وخطوط نقل ومرافق تخزين وتصدير. وهذا الفرق من أدق ما في المادة (7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>اتفاقية الامتياز</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>نفاذ ومدة</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>يُعمل بالنظام:</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>بعد مضي مائة وثمانين يوماً
-من تاريخ نشره مباشرة
-بعد مضي تسعين يوماً من تاريخ نشره في الجريدة الرسمية
-بعد صدور لائحته التنفيذية</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="inlineStr">
-        <is>
-          <t>بعد مضي تسعين يوماً من تاريخ نشره في الجريدة الرسمية</t>
-        </is>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>المادة (22)</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>مدة التهيئة هنا تسعون يوماً، وهي أقصر من المدة المعتادة في عدد من أنظمة القطاع والتي تبلغ مائة وثمانين يوماً.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>نظام المواد البترولية والبتروكيماوية</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>للحكومة بموجب اتفاقية الامتياز إعفاء الشركة من الريع كلياً أو جزئياً. في أي حال يكون هذا الإعفاء؟</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>إذا انخفض السعر العالمي للزيت الخام دون حد تحدده الحكومة ؛ إذا كانت اقتصاديات تطوير الحقل تستدعي ذلك، في الغاز الطبيعي وسوائل الغاز والمكثفات ؛ إذا كان الإنتاج موجهاً بكامله للاستهلاك المحلي ؛ إذا طلبت الشركة ذلك وأقره مجلس إدارتها</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>إذا كانت اقتصاديات تطوير الحقل تستدعي ذلك، في الغاز الطبيعي وسوائل الغاز والمكثفات</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>الفقرة (د) من المادة (7-1) من الاتفاقية</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>الإعفاء مقصور على الغاز وسوائله والمكثفات دون الزيت الخام، ومناطه اقتصاديات تطوير الحقل، ويكون للمدة التي تحددها الحكومة. فالريع هنا أداة سياسة طاقة لتحفيز تطوير حقول الغاز، لا مجرد مقابل مالي ثابت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>اتفاقية الامتياز</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>حد العقوبة</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>عقوبة من صدّر إلى خارج المملكة مادة بترولية مسعرة دون ترخيص أو شرع في ذلك تشمل:</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>الإنذار ثم الغرامة
-الغرامة فقط
-إلغاء الترخيص فقط
-السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="inlineStr">
-        <is>
-          <t>السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
-        </is>
-      </c>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>المادة (15)</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>هذه من أشد العقوبات في أنظمة قطاع الطاقة لأنها تمس الدعم الحكومي للمواد المسعرة، ولذلك جمعت بين السجن والغرامة والمصادرة، وجعلت الغرامة مرتبطة بقيمة المادة بالسعر العالمي.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>أي من الأنظمة التالية نص صراحة على عدم الإخلال بأحكام اتفاقية الامتياز فيما يتعلق بحق الشركة في نقل المواد الهيدروكربونية؟</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>نظام النقل البري على الطرق ؛ نظام الكهرباء ؛ نظام إمدادات الطاقة ؛ نظام المنافسة</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>نظام النقل البري على الطرق</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>البند (ثانياً) من المرسوم الملكي رقم (م/188) وتاريخ 1446/8/24هـ</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>تكرر في أكثر من نظام لاحق النص على عدم الإخلال بأحكام الاتفاقية، ومنه أيضاً نظام القياس والمعايرة. وهذا يبين أن الاتفاقية تُعامل بوصفها التزاماً قائماً تراعيه التشريعات الجديدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>اتفاقية الامتياز</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>الأول (تأسيسي)</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>أداة نظامية</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>صُدِّقت اتفاقية الامتياز بموجب:</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>المرسوم الملكي رقم (م/56) وتاريخ 1426/10/20هـ
-قرار مجلس الوزراء رقم (262)
-المرسوم الملكي رقم (م/37) وتاريخ 1439/4/2هـ
-المرسوم الملكي رقم (م/38) وتاريخ 1439/4/6هـ</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>المرسوم الملكي رقم (م/38) وتاريخ 1439/4/6هـ</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>المرسوم الملكي رقم (م/38) وتاريخ 1439/4/6هـ</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>صدرت الاتفاقية بعد أيام من صدور نظام المواد الهيدروكربونية بالمرسوم رقم (م/37)، وهذا الترتيب مقصود لأن النظام وضع الإطار السيادي والاتفاقية طبقته على أكبر مرخص له.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>اتفاقية الامتياز</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>المتوسط</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>نسبة</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>معدل الريع المستحق على إنتاج الزيت الخام والمكثفات بعد تعديل الاتفاقية هو:</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>عشرون في المائة
-خمسة عشر في المائة
-خمسة وعشرون في المائة
-اثنا عشر ونصف في المائة</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>خمسة عشر في المائة</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>الفقرة (أ) من المادة (7-1) من الاتفاقية بعد تعديلها</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>كان المعدل عشرين في المائة ثم خُفض إلى خمسة عشر في المائة بموجب تعديل الاتفاقية، وأجري تعديل مقابل في المادة (2-4)(أ)(1) من ملحق الاتفاقية. فالتعديل طال النص الأصلي والملحق معاً.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>اتفاقية الامتياز</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>استثناء</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>أي مما يلي لا يُستحق عليه ريع بموجب اتفاقية الامتياز؟</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="inlineStr">
-        <is>
-          <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها
-سوائل الغاز المباعة للغير
-الزيت الخام الذي تستخدمه الشركة في عملياتها
-المكثفات المنتجة</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>الفقرتان (أ) و(ب) من المادة (7-1) من الاتفاقية</t>
-        </is>
-      </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>الاتفاقية فرّقت بين الزيت والغاز في معاملة الاستخدام الذاتي: ريع الزيت الخام والمكثفات يشمل ما تستخدمه الشركة في عملياتها، أما الغاز وسوائله فلا ريع على ما يُستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها من معامل وخطوط نقل ومرافق تخزين وتصدير. وهذا الفرق من أدق ما في المادة (7).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>اتفاقية الامتياز</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>المتقدم</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>علاقة نظامية</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>العلاقة بين اتفاقية الامتياز ونظام المواد الهيدروكربونية هي:</t>
         </is>
       </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>الاتفاقية أعلى من النظام ولا تخضع له ؛ النظام لا ينطبق على الشركة لأنها مملوكة للدولة ؛ الاتفاقية ألغت النظام فيما يخص الشركة ؛ الاتفاقية رخصة تخضع لأحكام النظام، والنظام يحتفظ للدولة بالسلطة السيادية في اتخاذ قرار الإنتاج</t>
+        </is>
+      </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>الاتفاقية أعلى من النظام ولا تخضع له
-النظام لا ينطبق على الشركة لأنها مملوكة للدولة
-الاتفاقية ألغت النظام فيما يخص الشركة
-الاتفاقية رخصة تخضع لأحكام النظام، والنظام يحتفظ للدولة بالسلطة السيادية في اتخاذ قرار الإنتاج</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
           <t>الاتفاقية رخصة تخضع لأحكام النظام، والنظام يحتفظ للدولة بالسلطة السيادية في اتخاذ قرار الإنتاج</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>البند (ثانياً) من المرسوم الملكي رقم (م/37)، مع المادتين (7) و(9) من نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>نص المرسوم على سريان أي امتياز ممنوح قبل النفاذ وخضوعه لأحكام النظام، ومنع النظام غير الدولة من اتخاذ قرار الإنتاج ورتب البطلان على المخالفة. فالامتياز لا يعطي صاحبه سلطة على حجم الإنتاج.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1807,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1815,7 +1598,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>طريقة تعبئة بنك الأسئلة</t>
         </is>
@@ -1827,100 +1610,88 @@
       <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>الخيارات</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>كل خيار في سطر مستقل داخل الخلية نفسها (Alt + Enter في ويندوز، أو Option + Enter في ماك).</t>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>تُفصل الخيارات بالفاصلة المنقوطة العربية (؛) أو يُكتب كل خيار في سطر مستقل داخل الخلية نفسها.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>الإجابة الصحيحة</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>تُنسخ حرفياً من أحد الخيارات، فأي اختلاف ولو في مسافة أو حركة يوقف التحديث مع رسالة توضح رقم الصف.</t>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>تُنسخ حرفياً من أحد الخيارات، فأي اختلاف ولو في حرف أو حركة يوقف التحديث مع رسالة توضح رقم الصف.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>المستوى</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>إحدى القيم: الأول (تأسيسي)، المتوسط، المتقدم. لا يظهر المستوى للمشارك، ويُستخدم لترتيب الأسئلة من الأسهل إلى الأصعب.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>رقم فريد لكل سؤال، ويظهر في جدول النتائج (عمود الأسئلة الخاطئة) للرجوع إلى السؤال.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>النظام</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>يُجمع على أساسه السؤال في نتيجة المشارك حسب النظام.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>محور القياس</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>للاستخدام الداخلي ولا يُنشر في الموقع.</t>
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>أسئلة صح/خطأ</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>اكتب الخيارين: صح ؛ خطأ</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>أسئلة صح/خطأ</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>اكتب الخيارين: صح وخطأ في سطرين.</t>
-        </is>
-      </c>
+      <c r="A9" s="15" t="inlineStr"/>
+      <c r="B9" s="16" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr"/>
-      <c r="B10" s="19" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>تحديث الموقع</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>ارفع الملف إلى المستودع على GitHub باسم data/questions.xlsx (Add file ← Upload files)، فيتحدث الموقع تلقائياً خلال دقائق.</t>
         </is>

</xml_diff>

<commit_message>
Base development advice on knowledge types as well as regulations
Each question now carries a knowledge type (new spreadsheet column
نوع المعرفة: الاختصاص، المدد والإجراءات، الحدود والعقوبات، المفاهيم
والتعريفات، نطاق الأنظمة والعلاقة بينها، القيود والاستثناءات). The
results page lists every type scored below 75% with concrete study
advice, the regulations where the mistakes happened and the legal
references of the missed questions; per-regulation advice becomes a
short line each. Advice text per type lives in config.js.

Results now include by_skill. A results table without that column
rejects the row, so the site resends it without by_skill and collection
keeps working until the column is added (SQL in tools/supabase-setup.sql).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdJRTf8G26dx7ZenTkKWdk
</commit_message>
<xml_diff>
--- a/data/questions.xlsx
+++ b/data/questions.xlsx
@@ -11,7 +11,7 @@
     <sheet name="طريقة التعبئة" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بنك الأسئلة'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بنك الأسئلة'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F5C99"/>
       <sz val="10"/>
     </font>
     <font>
@@ -110,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -127,6 +132,9 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
@@ -137,6 +145,9 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -151,7 +162,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
@@ -523,17 +537,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -554,25 +569,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>نوع المعرفة</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>السؤال</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>الخيارات</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>الإجابة الصحيحة</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>السند النظامي</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>شرح مبسط</t>
         </is>
@@ -592,27 +612,32 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>الاختصاص</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>لا يُعد من مهام الهيئة السعودية لتنظيم الكهرباء:</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>إصدار اللوائح التنفيذية ؛ البت في الشكاوى المتعلقة بنشاط الكهرباء ؛ إعداد السياسات والاستراتيجيات الوطنية لقطاع الكهرباء</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>إعداد السياسات والاستراتيجيات الوطنية لقطاع الكهرباء</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>الفقرة (1) من المادة (3) في اختصاص الوزارة، مقابل المادة (4) في اختصاص الهيئة</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>إعداد السياسات والاستراتيجيات والرفع بها لاعتمادها اختصاص أصيل للوزارة، بينما تعمل الهيئة في ضوء تلك السياسات المعتمدة. وهذا السؤال يقيس التفريق بين دور صانع السياسة ودور المنظم.</t>
         </is>
@@ -632,307 +657,347 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>المفاهيم والتعريفات</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>الفرق بين "التعريفة" و"السعر" في نظام الكهرباء أن:</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>التعريفة مقابل مالي معتمد، والسعر مقابل يُتفق عليه بين مرخص لهما أو بين مرخص له ومستهلك كبير ؛ التعريفة تشمل الضريبة والسعر لا يشملها ؛ التعريفة سنوية والسعر يراجع شهرياً ؛ التعريفة للمستهلك المنزلي والسعر للمستهلك التجاري</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>التعريفة مقابل مالي معتمد، والسعر مقابل يُتفق عليه بين مرخص لهما أو بين مرخص له ومستهلك كبير</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>المادة (1) - تعريفا التعريفة والسعر، مع الفقرة (3) من المادة (12)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>التعريفة معتمدة وتسري على فئات المستهلكين، والسعر ثمرة تفاوض تجاري مباشر يجوز أن يختلف عن التعريفة المعتمدة وفق ما تحدده اللوائح. ولهذا ارتبط وصف المستهلك الكبير بأثر عملي، وهو إمكان التعاقد بسعر خارج التعريفة.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>المدد والإجراءات</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>تتخذ الهيئة السعودية لتنظيم الكهرباء إجراءات عاجلة بحق المخالف مثل:</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>إيقاف مزاولة نشاط الكهرباء جزئياً أو كلياً لمدة لا تتجاوز سنة ؛ إلغاء الرخصة ؛ إيقاف مزاولته للنشاط جزئياً أو كلياً بما لا يتجاوز (6) أشهر</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>إيقاف مزاولته للنشاط جزئياً أو كلياً بما لا يتجاوز (6) أشهر</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (ج) من الفقرة (1) من المادة (20)، مقابل الفقرة (1) من المادة (18)</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>يفرق النظام بين إجراء عاجل تتخذه الهيئة بقرار من المحافظ أو من ينيبه ومدته لا تتجاوز ستة أشهر، وبين عقوبة توقعها اللجنة بعد النظر في المخالفة وتصل إلى إيقاف سنة أو إلغاء الرخصة أو غرامة. والخياران الآخران عقوبات لا إجراءات عاجلة.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>الحدود والعقوبات</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>يجب على المرخص له الحصول على موافقة الهيئة قبل شراء أسهم مرخص له آخر إذا بلغت النسبة:</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>(10%) عشرة في المائة أو أكثر ؛ (20%) عشرين في المائة أو أكثر ؛ أي نسبة مهما قلّت ؛ (5%) خمسة في المائة أو أكثر، أو نسبة أقل إذا أدت إلى إنشاء وضع مهيمن</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>(5%) خمسة في المائة أو أكثر، أو نسبة أقل إذا أدت إلى إنشاء وضع مهيمن</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>الفقرة (5) من المادة (13)، مع تعريف الوضع المهيمن في المادة (1)</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>العتبة الرقمية خمسة في المائة، ومعها عتبة وصفية مؤداها أن النسبة الأقل تحتاج موافقة كذلك متى أدت إلى إنشاء وضع مهيمن في أي جزء من الأنشطة الكهربائية. والوضع المهيمن معرّف بأنه امتلاك القدرة على التأثير في عدالة اتخاذ القرارات أو التنافس المشروع.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>نظام الكهرباء</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>المدد والإجراءات</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>إذا رفضت الهيئة إصدار رخصة لشخص استوفى جميع الشروط، أو مضى (30) يوم عمل من تاريخ اكتمال طلبه دون البت فيه، فله الحق النظامي في:</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>التظلم أمام المحكمة التجارية ؛ التظلم أمام المحكمة الإدارية ؛ الاعتراض أمام الهيئة السعودية لتنظيم الكهرباء</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>التظلم أمام المحكمة الإدارية</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>الفقرة (4) من المادة (5)</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>أوجب النظام إصدار الرخصة خلال ثلاثين يوم عمل من اكتمال الطلب متى توافرت الشروط، واشترط تسبيب قرار الرفض، وأتاح لمن رفض طلبه أو مضت المدة دون بت التظلم أمام المحكمة الإدارية. والسبب أن القرار قرار إداري لا نزاع تجاري.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>الاختصاص</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>الجهة المختصة بإصدار رخص مزاولة أوجه النشاط بعد تعديل النظام هي:</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>هيئة تنظيم المياه والكهرباء ؛ وزارة الطاقة ؛ وزارة الصناعة والثروة المعدنية ؛ الهيئة العامة للنقل</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>وزارة الطاقة</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>المادة (3) بعد تعديلها بالمرسوم الملكي رقم (م/112) وتاريخ 1443/11/9هـ</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>صدر النظام سنة 1438 وأسند الاختصاص إلى الهيئة، ثم نقله التعديل إلى الوزارة بإحلال كلمة الوزارة محل الهيئة. ولهذا يجب الرجوع إلى النص المعدل لا الأصلي عند تحديد الجهة المختصة.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>الحدود والعقوبات</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>تُعد في حكم المستهلك التجاري المنشآت الصناعية الصغيرة التي لا يتجاوز استهلاكها للغاز الجاف:</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>(176.500) قدم مكعب يومياً ؛ (100.000) قدم مكعب يومياً ؛ (500.000) قدم مكعب يومياً ؛ (250.000) قدم مكعب يومياً</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>(176.500) قدم مكعب يومياً</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>المادة (1) - تعريف المستهلك التجاري</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>الحد رقم منصوص عليه في التعريف نفسه لا تحدده اللوائح، وأثره أن المنشأة الصناعية الصغيرة دون هذا الحد تعامل معاملة المستهلك التجاري وتخضع لهذا النظام، وما تجاوزه يخرج إلى منظومة تخصيص الطاقة.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>المدد والإجراءات</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>تقدم مرخص له بطلب موافقة على نقل ملكية أصول أساسية، ومضت تسعون يوماً من تاريخ اكتمال الطلب دون بت. الأثر النظامي:</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>يُعد مضي المدة إذناً له بالتصرف ؛ يُعد الطلب مرفوضاً ضمناً ؛ يجب عليه التقدم بطلب جديد ؛ يُحال الطلب إلى اللجنة للنظر فيه</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>يُعد مضي المدة إذناً له بالتصرف</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>المادة (13) بعد تعديلها بالمرسوم الملكي رقم (م/112)</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>المدة تسعون يوماً من اكتمال الطلب، ورتب النظام على مضيها دون بت أثراً إيجابياً هو الإذن بالتصرف لا الرفض الضمني. ويجب أن يكون قرار الرفض مسبباً. والأصول الأساسية هي ما يترتب على نقل ملكيتها إخلال بأداء النشاط المرخص به، ومنها شبكة توزيع الغاز الجاف ومرافق غاز البترول السائل.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>الحدود والعقوبات</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>الحد الأعلى للغرامة على مخالفة أحكام نظام توزيع الغاز الجاف وغاز البترول السائل هو:</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>عشرة ملايين ريال ؛ خمسة ملايين ريال ؛ ثلاثون مليون ريال ؛ عشرون مليون ريال</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>خمسة ملايين ريال</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (أ) من الفقرة (1) من المادة (16)</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>سقف الغرامة هنا خمسة ملايين، ويجوز أن يقترن بإيقاف النشاط جزئياً أو كلياً لمدة لا تتجاوز سنة أو بإلغاء الرخصة. ويفيد استحضار الأسقف في أنظمة القطاع معاً: نظام الكهرباء عشرة ملايين، وإمدادات الطاقة عشرون مليوناً، وجريمة تصدير المادة البترولية المسعرة ثلاثون مليوناً أو ضعفا قيمتها أيهما أعلى.</t>
         </is>
@@ -952,387 +1017,437 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>المفاهيم والتعريفات</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>أي وصف نظامي يلحق ملكية الدولة للموارد الهيدروكربونية؟</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>غير قابلة للتصرف ولا تسقط بالتقادم ؛ تنتقل إلى المرخص له بانتهاء مدة الرخصة ؛ تسقط بالتقادم الطويل إذا لم تستغل ؛ قابلة للتصرف بموافقة مجلس الوزراء</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>غير قابلة للتصرف ولا تسقط بالتقادم</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>المادة (5) مع المادة (4)</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>حصّن النظام ملكية الدولة بوصفين معاً: عدم قابليتها للتصرف، وعدم سقوطها بالتقادم، فلا يكسب أحد حقاً عليها بطول وضع اليد ولا بتصرف يقع من أي جهة. ويسند ذلك أن للدولة سيادة دائمة على هذه الموارد تمارسها بما يحقق مصلحتها وأمنها وتنميتها الاقتصادية.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>المفاهيم والتعريفات</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>تنتقل ملكية المواد الهيدروكربونية من الدولة إلى المرخص له عند:</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>توقيع الرخصة ؛ سداد الريع المستحق عن الكمية المنتجة ؛ تصدير المنتج خارج الإقليم ؛ رأس البئر، أو عند استخلاصها في منشأة معالجة لتحصيل منتجات القطران الطبيعي ورمال القار وما في حكمها</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>رأس البئر، أو عند استخلاصها في منشأة معالجة لتحصيل منتجات القطران الطبيعي ورمال القار وما في حكمها</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>المادة (3)</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>النظام حدد نقطة زمنية ومكانية لانتقال الملكية، وهي رأس البئر في الحالة المعتادة، أو لحظة الاستخلاص في منشأة المعالجة في حالات القطران الطبيعي وأحجار أو رمال القار وغيرها من مواد الصخور. وقبل هذه النقطة المادة ملك للدولة، فالرخصة تمنح حق ممارسة العمليات لا ملكية الثروة في باطن الأرض.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>المفاهيم والتعريفات</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>المقصود بـ "قرار الإنتاج" في النظام هو:</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>قرار يصدر عن منظمة أوبك وتلتزم به المملكة ؛ خطة تشغيلية سنوية يعدها المرخص له ؛ قرار تجاري تتخذه الشركة المنتجة بحسب أسعار السوق ؛ أمر أو توجيه مكتوب من الدولة يضع الحد الأقصى للإنتاج أو يحدد مستوى الطاقة الإنتاجية القصوى المستدامة</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>أمر أو توجيه مكتوب من الدولة يضع الحد الأقصى للإنتاج أو يحدد مستوى الطاقة الإنتاجية القصوى المستدامة</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>المادة (1) - التعريفات، والمادة (7)</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>قرار الإنتاج أداة سيادية لا تجارية، وتراعي الدولة عند اتخاذه اعتبارات التنمية الاقتصادية والبيئة والأمن الوطني والسياسة الخارجية والاحتياجات المحلية للطاقة والمصلحة العامة.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>القيود والاستثناءات</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>متى يُمنع المرخص له من بيع مادة هيدروكربونية أو مشتق منها حصل عليه بموجب الرخصة؟</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>إذا كان المشتري شخصاً أجنبياً ؛ إذا خالف البيع ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا للدولة في وقت الحرب أو في الحالات الطارئة في العلاقات الدولية ؛ إذا لم تصادق الوزارة على عقد البيع مسبقاً ؛ إذا قل سعر البيع عن السعر العالمي وقت التعاقد</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>إذا خالف البيع ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا للدولة في وقت الحرب أو في الحالات الطارئة في العلاقات الدولية</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>نص النظام في شأن قيد البيع لحماية مصالح الأمن العليا للدولة</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="I14" s="13" t="inlineStr">
         <is>
           <t>القيد استثنائي ومربوط بحالتين: وقت الحرب، والحالات الطارئة في العلاقات الدولية، ومناطه ما تقرره الحكومة ضرورياً لحماية مصالح الأمن العليا. فهو ليس قيداً على هوية المشتري ولا على السعر ولا رقابة مسبقة على العقود.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>الاختصاص</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>أي مما يلي لا يُعد من مهام لجنة تخصيص الطاقة؟</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>اعتماد معايير تخصيص الطاقة التي تقترحها الوزارة ؛ إعداد لائحة التخصيص واقتراح تعديلها ؛ مراجعة معايير التخصيص كل ثلاث سنوات أو حسب الحاجة ؛ إصدار وثيقة تخصيص الطاقة للمستهلك</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>إصدار وثيقة تخصيص الطاقة للمستهلك</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>الفقرة (3) من المادة (3)، مقابل المادة (4)</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>اللجنة جهة معايير وسياسات، أما الإصدار الفعلي لوثيقة التخصيص فتقوم به الوزارة بناءً على الطاقة المتاحة والمعايير المعتمدة من اللجنة. والتفريق بين من يضع المعيار ومن يطبقه هو مربط السؤال.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>نطاق الأنظمة والعلاقة بينها</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>أي مما يلي لا يدخل ضمن الأنشطة التي يشترط لها ترخيص من الوزارة بموجب نظام إمدادات الطاقة؟</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>تنقية الغاز ؛ تكرير الزيت الخام ؛ تجميع الغاز الطبيعي وسوائله ؛ التوزيع المحلي للغاز الطبيعي وسوائله</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>تكرير الزيت الخام</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>الفقرة (1) من المادة (5)، مقابل الفقرة (1) من المادة (2)</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="I16" s="13" t="inlineStr">
         <is>
           <t>الترخيص في هذا النظام مقصور على أنشطة الغاز الطبيعي وسوائله والأنشطة المتعلقة بالهيدروجين، وتشمل النقل والمعالجة والتجزئة وتنقية الغاز والتجميع والتخزين والتوزيع المحلي والاستيراد والتصدير والبيع وإنشاء وتملك وتشغيل الشبكات والمرافق. أما تكرير الزيت الخام فهو مجال من مجالات تخصيص الطاقة لا نشاط مرخص بهذا النظام، وتحكمه منظومة المواد البترولية والبتروكيماوية.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>المدد والإجراءات</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>يشترط الحصول على وثيقة تخصيص الطاقة من الوزارة:</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>قبل صدور موافقة الجهة المشرفة بممارسة النشاط الذي يتطلب تخصيصاً للطاقة ؛ بعد بدء التشغيل الفعلي ؛ عند تجديد السجل التجاري ؛ عند تصدير المنتج إلى خارج المملكة</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>قبل صدور موافقة الجهة المشرفة بممارسة النشاط الذي يتطلب تخصيصاً للطاقة</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>المادة (6)</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>جعل النظام وثيقة التخصيص شرطاً سابقاً على موافقة الجهة المشرفة، حتى لا تُمنح تراخيص لمشاريع لا تتوافر لها طاقة مخصصة. وهذا من أهم الآثار العملية للنظام على المستثمرين.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>الحدود والعقوبات</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>الحد الأعلى للغرامة على مخالفة أحكام النظام أو اللوائح أو لائحة التخصيص أو التراخيص هو:</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>عشرة ملايين ريال ؛ عشرون مليون ريال ؛ ثلاثون مليون ريال ؛ خمسة ملايين ريال</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>عشرون مليون ريال</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="H18" s="13" t="inlineStr">
         <is>
           <t>الفقرة الفرعية (أ) من الفقرة (1) من المادة (8)</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="I18" s="13" t="inlineStr">
         <is>
           <t>تصل الغرامة إلى عشرين مليون ريال، ويجوز معها إيقاف الترخيص جزئياً أو كلياً لمدة لا تتجاوز سنة، أو إلغاؤه. ويقابل ذلك سقف مماثل لمخالفة وثيقة التخصيص.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>نطاق الأنظمة والعلاقة بينها</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>أي نظام يحكم نقل المواد البترولية وتخزينها واستيرادها وتصديرها؟</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>نظام إمدادات الطاقة ؛ نظام المواد البترولية والبتروكيماوية ؛ نظام المواد الهيدروكربونية ؛ نظام توزيع الغاز الجاف وغاز البترول السائل</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>المادة (1) - تعريف العمليات البترولية، مقابل المادة (1) من نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>النظامان يقتسمان سلسلة القيمة: المواد الهيدروكربونية يحكم المنبع من مسح وكشف وتنقيب وحفر وتقييم وتطوير واستخراج وإنتاج ومعالجة، والمواد البترولية والبتروكيماوية يحكم المصب من استخدام وبيع وشراء ونقل وتخزين واستيراد وتصدير وتعبئة، ويدخل فيه إنشاء أو تشغيل مصفاة تكرير أو فرضة أو محطة توزيع. وتحديد النظام الحاكم هو أول ما يُسأل عنه المستشار في أي معاملة.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>نطاق الأنظمة والعلاقة بينها</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>النظام الذي حل محله نظام المواد البترولية والبتروكيماوية هو:</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>نظام المواد الهيدروكربونية ؛ نظام التجارة بالمنتجات البترولية ؛ نظام إمدادات الغاز وتسعيره ؛ نظام الكهرباء</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>نظام التجارة بالمنتجات البترولية</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>المادة (21)</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>حل النظام محل نظام التجارة بالمنتجات البترولية الصادر في 28 محرم 1439هـ، وألغى ما يتعارض معه من أحكام. أما نظام المواد الهيدروكربونية فباق ويغطي مرحلة المنبع.</t>
         </is>
@@ -1352,234 +1467,264 @@
           <t>الأول (تأسيسي)</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>المفاهيم والتعريفات</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>أي مما يلي لا يدخل ضمن العمليات البترولية كما عرفها النظام؟</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>تخزين المواد البترولية أو استيرادها أو تصديرها ؛ بيع المواد البترولية أو شراؤها أو نقلها ؛ التنقيب عن الزيت الخام واستخراجه ؛ إنشاء أو تشغيل مصفاة تكرير أو محطة توزيع</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>التنقيب عن الزيت الخام واستخراجه</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>المادة (1) - تعريف العمليات البترولية</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>العمليات البترولية في هذا النظام تقع في المصب: الاستخدام والبيع والشراء والنقل والتخزين والاستيراد والتصدير والتعبئة والمعالجة وإنشاء المصافي والفرض ومحطات التوزيع. أما التنقيب والاستخراج فمحلهما نظام المواد الهيدروكربونية.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>نظام المواد البترولية والبتروكيماوية</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>الحدود والعقوبات</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>عقوبة من صدّر إلى خارج المملكة مادة بترولية مسعرة دون ترخيص أو شرع في ذلك تشمل:</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>الإنذار ثم الغرامة ؛ الغرامة فقط ؛ إلغاء الترخيص فقط ؛ السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>السجن مدة لا تتجاوز خمس سنوات وغرامة لا تتجاوز ثلاثين مليون ريال أو ضعفي قيمة المادة بالسعر العالمي أيهما أعلى ومصادرة المضبوطات</t>
         </is>
       </c>
-      <c r="G22" s="11" t="inlineStr">
+      <c r="H22" s="13" t="inlineStr">
         <is>
           <t>المادة (15)</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="I22" s="13" t="inlineStr">
         <is>
           <t>هذه من أشد العقوبات في أنظمة قطاع الطاقة لأنها تمس الدعم الحكومي للمواد المسعرة، ولذلك جمعت بين السجن والغرامة والمصادرة، وجعلت الغرامة مرتبطة بقيمة المادة بالسعر العالمي.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>اتفاقية الامتياز</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>القيود والاستثناءات</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>أي مما يلي لا يُستحق عليه ريع بموجب اتفاقية الامتياز؟</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها ؛ سوائل الغاز المباعة للغير ؛ الزيت الخام الذي تستخدمه الشركة في عملياتها ؛ المكثفات المنتجة</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>الغاز الطبيعي وسوائله المستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr">
         <is>
           <t>الفقرتان (أ) و(ب) من المادة (7-1) من الاتفاقية</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>الاتفاقية فرّقت بين الزيت والغاز في معاملة الاستخدام الذاتي: ريع الزيت الخام والمكثفات يشمل ما تستخدمه الشركة في عملياتها، أما الغاز وسوائله فلا ريع على ما يُستخدم في عمليات الإنتاج والتنقيب وما يرتبط بها من معامل وخطوط نقل ومرافق تخزين وتصدير. وهذا الفرق من أدق ما في المادة (7).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>اتفاقية الامتياز</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>المتوسط</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>القيود والاستثناءات</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>للحكومة بموجب اتفاقية الامتياز إعفاء الشركة من الريع كلياً أو جزئياً. في أي حال يكون هذا الإعفاء؟</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>إذا انخفض السعر العالمي للزيت الخام دون حد تحدده الحكومة ؛ إذا كانت اقتصاديات تطوير الحقل تستدعي ذلك، في الغاز الطبيعي وسوائل الغاز والمكثفات ؛ إذا كان الإنتاج موجهاً بكامله للاستهلاك المحلي ؛ إذا طلبت الشركة ذلك وأقره مجلس إدارتها</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>إذا كانت اقتصاديات تطوير الحقل تستدعي ذلك، في الغاز الطبيعي وسوائل الغاز والمكثفات</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>الفقرة (د) من المادة (7-1) من الاتفاقية</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>الإعفاء مقصور على الغاز وسوائله والمكثفات دون الزيت الخام، ومناطه اقتصاديات تطوير الحقل، ويكون للمدة التي تحددها الحكومة. فالريع هنا أداة سياسة طاقة لتحفيز تطوير حقول الغاز، لا مجرد مقابل مالي ثابت.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>اتفاقية الامتياز</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>نطاق الأنظمة والعلاقة بينها</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t>أي من الأنظمة التالية نص صراحة على عدم الإخلال بأحكام اتفاقية الامتياز فيما يتعلق بحق الشركة في نقل المواد الهيدروكربونية؟</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>نظام النقل البري على الطرق ؛ نظام الكهرباء ؛ نظام إمدادات الطاقة ؛ نظام المنافسة</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr">
         <is>
           <t>نظام النقل البري على الطرق</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>البند (ثانياً) من المرسوم الملكي رقم (م/188) وتاريخ 1446/8/24هـ</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="I25" s="13" t="inlineStr">
         <is>
           <t>تكرر في أكثر من نظام لاحق النص على عدم الإخلال بأحكام الاتفاقية، ومنه أيضاً نظام القياس والمعايرة. وهذا يبين أن الاتفاقية تُعامل بوصفها التزاماً قائماً تراعيه التشريعات الجديدة.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>اتفاقية الامتياز</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>المتقدم</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>نطاق الأنظمة والعلاقة بينها</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>العلاقة بين اتفاقية الامتياز ونظام المواد الهيدروكربونية هي:</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>الاتفاقية أعلى من النظام ولا تخضع له ؛ النظام لا ينطبق على الشركة لأنها مملوكة للدولة ؛ الاتفاقية ألغت النظام فيما يخص الشركة ؛ الاتفاقية رخصة تخضع لأحكام النظام، والنظام يحتفظ للدولة بالسلطة السيادية في اتخاذ قرار الإنتاج</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>الاتفاقية رخصة تخضع لأحكام النظام، والنظام يحتفظ للدولة بالسلطة السيادية في اتخاذ قرار الإنتاج</t>
         </is>
       </c>
-      <c r="G26" s="11" t="inlineStr">
+      <c r="H26" s="13" t="inlineStr">
         <is>
           <t>البند (ثانياً) من المرسوم الملكي رقم (م/37)، مع المادتين (7) و(9) من نظام المواد الهيدروكربونية</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="I26" s="13" t="inlineStr">
         <is>
           <t>نص المرسوم على سريان أي امتياز ممنوح قبل النفاذ وخضوعه لأحكام النظام، ومنع النظام غير الدولة من اتخاذ قرار الإنتاج ورتب البطلان على المخالفة. فالامتياز لا يعطي صاحبه سلطة على حجم الإنتاج.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1590,7 +1735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1598,7 +1743,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>طريقة تعبئة بنك الأسئلة</t>
         </is>
@@ -1610,88 +1755,100 @@
       <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>الخيارات</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>تُفصل الخيارات بالفاصلة المنقوطة العربية (؛) أو يُكتب كل خيار في سطر مستقل داخل الخلية نفسها.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>الإجابة الصحيحة</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>تُنسخ حرفياً من أحد الخيارات، فأي اختلاف ولو في حرف أو حركة يوقف التحديث مع رسالة توضح رقم الصف.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>المستوى</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>إحدى القيم: الأول (تأسيسي)، المتوسط، المتقدم. لا يظهر المستوى للمشارك، ويُستخدم لترتيب الأسئلة من الأسهل إلى الأصعب.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>رقم فريد لكل سؤال، ويظهر في جدول النتائج (عمود الأسئلة الخاطئة) للرجوع إلى السؤال.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>النظام</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>يُجمع على أساسه السؤال في نتيجة المشارك حسب النظام.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>نوع المعرفة</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>نوع المعرفة التي يقيسها السؤال (مثل: الاختصاص، المدد والإجراءات). تُبنى عليه توصيات التطوير، ونص كل توصية في ملف config.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>أسئلة صح/خطأ</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>اكتب الخيارين: صح ؛ خطأ</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr"/>
-      <c r="B9" s="16" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr"/>
+      <c r="B10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>تحديث الموقع</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>ارفع الملف إلى المستودع على GitHub باسم data/questions.xlsx (Add file ← Upload files)، فيتحدث الموقع تلقائياً خلال دقائق.</t>
         </is>

</xml_diff>